<commit_message>
Ball tracking: template tracking, tiled detection, feet-anchored gaps
- Template matching follows the ball through motion blur with
  forward/backward agreement verification (24 frames recovered)
- Native-resolution tiled detection sweeps frames the detector missed
  (110/121 blind frames recovered, physics-gated before acceptance)
- Gaps that start and end at players' feet anchor the marker to the
  nearest player instead of gliding across grass
- Real-detection coverage: 600 -> 666 of 750 frames; longest blind
  gap down from 24 to 9 frames
</commit_message>
<xml_diff>
--- a/output_videos/player_ratings.xlsx
+++ b/output_videos/player_ratings.xlsx
@@ -443,7 +443,7 @@
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="15" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="60" customWidth="1" min="27" max="27"/>
+    <col width="58" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,7 +690,7 @@
         <v>20</v>
       </c>
       <c r="G3" t="n">
-        <v>7.63</v>
+        <v>7.62</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
@@ -755,27 +755,27 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B4" t="n">
         <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>defender</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>0.5</v>
       </c>
       <c r="E4" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="G4" t="n">
-        <v>7.39</v>
+        <v>6.83</v>
       </c>
       <c r="H4" t="n">
         <v>100</v>
@@ -784,7 +784,7 @@
         <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -817,7 +817,7 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
@@ -826,43 +826,43 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>65.3</v>
+        <v>52.5</v>
       </c>
       <c r="Y4" t="n">
-        <v>130.6</v>
+        <v>105</v>
       </c>
       <c r="Z4" t="n">
         <v>750</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2x Short pass; 1x Challenge won; 1x Won in own third; 1x Link up</t>
+          <t>1x Short pass; 1x Challenge won</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" t="n">
         <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>midfielder</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>0.5</v>
       </c>
       <c r="E5" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="F5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>6.83</v>
+        <v>6.5</v>
       </c>
       <c r="H5" t="n">
         <v>100</v>
@@ -871,7 +871,7 @@
         <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -889,7 +889,7 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -913,52 +913,50 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>52.5</v>
+        <v>50.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>105</v>
+        <v>100.6</v>
       </c>
       <c r="Z5" t="n">
         <v>750</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>1x Short pass; 1x Challenge won</t>
+          <t>2x Short pass; 1x Under pressure; 2x Challenge won</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>midfielder</t>
+          <t>defender</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.5</v>
+        <v>0.44</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>1.75</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
+        <v>39.83</v>
       </c>
       <c r="G6" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="H6" t="n">
         <v>100</v>
       </c>
-      <c r="I6" t="n">
-        <v>100</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -967,7 +965,7 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -976,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -994,32 +992,32 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>50.3</v>
+        <v>46.8</v>
       </c>
       <c r="Y6" t="n">
-        <v>100.6</v>
+        <v>106.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>750</v>
+        <v>659</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>3x Short pass; 1x Under pressure; 2x Challenge won</t>
+          <t>1x Short pass; 1x Dribble; 1x Pace (sprint)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1027,23 +1025,23 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.44</v>
+        <v>0.42</v>
       </c>
       <c r="E7" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="F7" t="n">
-        <v>39.83</v>
+        <v>59.62</v>
       </c>
       <c r="G7" t="n">
-        <v>5.76</v>
+        <v>6.09</v>
       </c>
       <c r="H7" t="n">
         <v>100</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1052,7 +1050,7 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1076,32 +1074,32 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>46.8</v>
+        <v>42.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>106.5</v>
+        <v>102.3</v>
       </c>
       <c r="Z7" t="n">
-        <v>659</v>
+        <v>629</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>1x Short pass; 1x Dribble; 1x Pace (sprint)</t>
+          <t>2x Short pass; 1x Under pressure; 1x Link up</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B8" t="n">
         <v>2</v>
@@ -1112,16 +1110,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
       <c r="E8" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>59.62</v>
+        <v>40</v>
       </c>
       <c r="G8" t="n">
-        <v>5.6</v>
+        <v>5.58</v>
       </c>
       <c r="H8" t="n">
         <v>100</v>
@@ -1137,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -1170,17 +1168,17 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>42.9</v>
+        <v>65.3</v>
       </c>
       <c r="Y8" t="n">
-        <v>102.3</v>
+        <v>130.6</v>
       </c>
       <c r="Z8" t="n">
-        <v>629</v>
+        <v>750</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2x Short pass; 1x Under pressure; 1x Link up</t>
+          <t>2x Short pass; 1x Link up</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1204,7 @@
         <v>20</v>
       </c>
       <c r="G9" t="n">
-        <v>5.13</v>
+        <v>5.25</v>
       </c>
       <c r="H9" t="n">
         <v>100</v>
@@ -1293,7 +1291,7 @@
         <v>30</v>
       </c>
       <c r="G10" t="n">
-        <v>4.69</v>
+        <v>4.88</v>
       </c>
       <c r="H10" t="n">
         <v>100</v>
@@ -1358,30 +1356,32 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>defender</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>0.5</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="G11" t="n">
-        <v>4.27</v>
+        <v>4.63</v>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1422,51 +1422,49 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>61</v>
+        <v>80.7</v>
       </c>
       <c r="Y11" t="n">
-        <v>122</v>
+        <v>161.4</v>
       </c>
       <c r="Z11" t="n">
         <v>750</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>no recorded actions</t>
+          <t>1x Pace (sprint) | bad: 1x Challenge lost</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>defender</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="D12" t="n">
         <v>0.5</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>3.88</v>
+        <v>4.27</v>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
         <v>0</v>
       </c>
@@ -1489,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -1507,53 +1505,51 @@
         <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>80.7</v>
+        <v>61</v>
       </c>
       <c r="Y12" t="n">
-        <v>161.4</v>
+        <v>122</v>
       </c>
       <c r="Z12" t="n">
         <v>750</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>1x Pace (sprint) | bad: 1x Challenge lost</t>
+          <t>no recorded actions</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>defender</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>0.5</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="H13" t="n">
-        <v>100</v>
-      </c>
+        <v>4.11</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1595,50 +1591,50 @@
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>45.5</v>
+        <v>59.1</v>
       </c>
       <c r="Y13" t="n">
-        <v>91</v>
+        <v>118.7</v>
       </c>
       <c r="Z13" t="n">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2x Short pass</t>
+          <t>no recorded actions</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>midfielder</t>
+          <t>defender</t>
         </is>
       </c>
       <c r="D14" t="n">
         <v>0.5</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>-0.25</v>
       </c>
       <c r="F14" t="n">
-        <v>20</v>
+        <v>-5</v>
       </c>
       <c r="G14" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="H14" t="n">
-        <v>100</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>4.06</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1647,7 +1643,7 @@
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1659,7 +1655,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1677,29 +1673,29 @@
         <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>52.5</v>
+        <v>66.2</v>
       </c>
       <c r="Y14" t="n">
-        <v>105</v>
+        <v>132.4</v>
       </c>
       <c r="Z14" t="n">
         <v>750</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>1x Short pass; 1x Under pressure</t>
+          <t>1x Pace (sprint) | bad: 1x Challenge lost</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1710,20 +1706,20 @@
         <v>0.5</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.25</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>-5</v>
+        <v>20</v>
       </c>
       <c r="G15" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
+        <v>3.72</v>
+      </c>
+      <c r="H15" t="n">
+        <v>100</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1744,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1762,51 +1758,53 @@
         <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>66.2</v>
+        <v>45.5</v>
       </c>
       <c r="Y15" t="n">
-        <v>132.4</v>
+        <v>91</v>
       </c>
       <c r="Z15" t="n">
         <v>750</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>1x Pace (sprint) | bad: 1x Challenge lost</t>
+          <t>2x Short pass</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>midfielder</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>0.5</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G16" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
+        <v>3.52</v>
+      </c>
+      <c r="H16" t="n">
+        <v>100</v>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1815,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -1848,30 +1846,30 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>50.8</v>
+        <v>52.5</v>
       </c>
       <c r="Y16" t="n">
-        <v>101.6</v>
+        <v>105</v>
       </c>
       <c r="Z16" t="n">
         <v>750</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>no recorded actions</t>
+          <t>1x Short pass; 1x Under pressure</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B17" t="n">
         <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>midfielder</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1884,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>3.22</v>
+        <v>3.3</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -1931,10 +1929,10 @@
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>58.2</v>
+        <v>50.8</v>
       </c>
       <c r="Y17" t="n">
-        <v>116.4</v>
+        <v>101.6</v>
       </c>
       <c r="Z17" t="n">
         <v>750</v>
@@ -1947,10 +1945,10 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1958,7 +1956,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -1967,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>3.13</v>
+        <v>3.22</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -2014,13 +2012,13 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>55.9</v>
+        <v>58.2</v>
       </c>
       <c r="Y18" t="n">
-        <v>115</v>
+        <v>116.4</v>
       </c>
       <c r="Z18" t="n">
-        <v>729</v>
+        <v>750</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -2030,18 +2028,18 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>defender</t>
+          <t>midfielder</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -2050,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>3.01</v>
+        <v>3.13</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -2100,10 +2098,10 @@
         <v>55.9</v>
       </c>
       <c r="Y19" t="n">
-        <v>111.8</v>
+        <v>115</v>
       </c>
       <c r="Z19" t="n">
-        <v>750</v>
+        <v>729</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -2113,32 +2111,30 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>defender</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>0.5</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>-10.04</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>2.49</v>
+        <v>3.04</v>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
         <v>0</v>
       </c>
@@ -2161,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2182,17 +2178,17 @@
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>59.1</v>
+        <v>55.9</v>
       </c>
       <c r="Y20" t="n">
-        <v>118.7</v>
+        <v>111.8</v>
       </c>
       <c r="Z20" t="n">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>no recorded actions | bad: 1x Challenge lost</t>
+          <t>no recorded actions</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2214,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1.98</v>
+        <v>2.02</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -2545,7 +2541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2554,7 +2550,7 @@
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -2848,7 +2844,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Short pass 21 -&gt; 16 (14px, gain -10px, under pressure)</t>
+          <t>Short pass 21 -&gt; 16 (8px, gain -8px, under pressure)</t>
         </is>
       </c>
     </row>
@@ -2972,16 +2968,16 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Short pass 20 -&gt; 16 (24px, gain +20px)</t>
+          <t>Short pass 20 -&gt; 16 (24px, gain +18px)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="B14" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -3004,7 +3000,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Short pass 16 -&gt; 17 (75px, gain +75px)</t>
+          <t>Short pass 16 -&gt; 17 (16px, gain +16px)</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3038,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B16" t="n">
         <v>17.4</v>
@@ -3068,7 +3064,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Short pass 17 -&gt; 18 (221px, gain -213px)</t>
+          <t>Short pass 17 -&gt; 18 (201px, gain -190px)</t>
         </is>
       </c>
     </row>
@@ -3100,48 +3096,48 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Short pass 18 -&gt; 20 (52px, gain +41px)</t>
+          <t>Short pass 18 -&gt; 20 (52px, gain -44px)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>482</v>
+        <v>542</v>
       </c>
       <c r="B18" t="n">
-        <v>19.3</v>
+        <v>21.7</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Short pass</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>20</v>
       </c>
       <c r="E18" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>20: +1.0 (Challenge won); 11: -0.5 (Challenge lost); 20: +0.5 (Won in own third)</t>
+          <t>20: +0.5 (Short pass)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>challenge: 20 won ball off 11 (scramble of 2 exchanges), in own third</t>
+          <t>Short pass 20 -&gt; 13 (4px, gain +2px)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>542</v>
+        <v>571</v>
       </c>
       <c r="B19" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -3149,31 +3145,31 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E19" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F19" t="n">
         <v>2</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>20: +0.5 (Short pass)</t>
+          <t>13: +0.5 (Short pass)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Short pass 20 -&gt; 13 (4px, gain +2px)</t>
+          <t>Short pass 13 -&gt; 18 (2px, gain +2px)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>571</v>
+        <v>597</v>
       </c>
       <c r="B20" t="n">
-        <v>22.8</v>
+        <v>23.9</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -3181,63 +3177,63 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E20" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F20" t="n">
         <v>2</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>13: +0.5 (Short pass)</t>
+          <t>18: +0.5 (Short pass)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Short pass 13 -&gt; 18 (2px, gain +2px)</t>
+          <t>Short pass 18 -&gt; 17 (13px, gain +12px)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>597</v>
+        <v>639</v>
       </c>
       <c r="B21" t="n">
-        <v>23.9</v>
+        <v>25.6</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Short pass</t>
+          <t>Challenge</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E21" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
         <v>2</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>18: +0.5 (Short pass)</t>
+          <t>17: +1.0 (Challenge won); 7: -0.5 (Challenge lost)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Short pass 18 -&gt; 17 (13px, gain +12px)</t>
+          <t>challenge: 17 won ball off 7 (scramble of 2 exchanges)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>629</v>
+        <v>652</v>
       </c>
       <c r="B22" t="n">
-        <v>25.2</v>
+        <v>26.1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -3255,115 +3251,115 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>17: +0.5 (Short pass)</t>
+          <t>17: +0.5 (Short pass); 17: +0.5 (Under pressure)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Short pass 17 -&gt; 22 (33px, gain -30px)</t>
+          <t>Short pass 17 -&gt; 22 (4px, gain -4px, under pressure)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>639</v>
+        <v>653</v>
       </c>
       <c r="B23" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Close control</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>17</v>
-      </c>
-      <c r="E23" t="n">
-        <v>7</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
         <v>2</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>17: +1.0 (Challenge won); 7: -0.5 (Challenge lost)</t>
+          <t>22: +0.5 (Close control)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>challenge: 17 won ball off 7 (scramble of 2 exchanges)</t>
+          <t>close control: 22 kept the ball under pressure from 7</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>652</v>
+        <v>672</v>
       </c>
       <c r="B24" t="n">
-        <v>26.1</v>
+        <v>26.9</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Short pass</t>
+          <t>Challenge</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
         <v>22</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>17: +0.5 (Short pass); 17: +0.5 (Under pressure)</t>
+          <t>2: +1.0 (Challenge won); 22: -0.5 (Challenge lost)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Short pass 17 -&gt; 22 (4px, gain -4px, under pressure)</t>
+          <t>challenge: 2 won ball off 22</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>653</v>
+        <v>688</v>
       </c>
       <c r="B25" t="n">
-        <v>26.1</v>
+        <v>27.5</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Close control</t>
+          <t>Short pass</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>22</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10</v>
+      </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>22: +0.5 (Close control)</t>
+          <t>2: +0.5 (Short pass)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>close control: 22 kept the ball under pressure from 7</t>
+          <t>Short pass 2 -&gt; 10 (15px, gain -15px)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>679</v>
+        <v>692</v>
       </c>
       <c r="B26" t="n">
-        <v>27.2</v>
+        <v>27.7</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -3371,84 +3367,20 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E26" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2: +1.0 (Challenge won); 22: -0.5 (Challenge lost)</t>
+          <t>19: +1.0 (Challenge won); 3: -0.5 (Challenge lost)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
-        <is>
-          <t>challenge: 2 won ball off 22</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>688</v>
-      </c>
-      <c r="B27" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Short pass</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" t="n">
-        <v>10</v>
-      </c>
-      <c r="F27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2: +0.5 (Short pass)</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Short pass 2 -&gt; 10 (15px, gain -15px)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>692</v>
-      </c>
-      <c r="B28" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Challenge</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>19</v>
-      </c>
-      <c r="E28" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>19: +1.0 (Challenge won); 3: -0.5 (Challenge lost)</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
         <is>
           <t>challenge: 19 won ball off 3 (scramble of 3 exchanges)</t>
         </is>

</xml_diff>